<commit_message>
chore: update filtered_output.xlsx via GitHub Actions
</commit_message>
<xml_diff>
--- a/data/filtered_output.xlsx
+++ b/data/filtered_output.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -479,264 +479,990 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>ETERNAL</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>177.28</v>
+        <v>285.2</v>
       </c>
       <c r="C2" t="n">
-        <v>177.9</v>
+        <v>289.7</v>
       </c>
       <c r="D2" t="n">
-        <v>176.04</v>
+        <v>283.9</v>
       </c>
       <c r="E2" t="n">
-        <v>176.72</v>
+        <v>286.35</v>
       </c>
       <c r="F2" t="n">
-        <v>9835632</v>
+        <v>19958107</v>
       </c>
       <c r="G2" t="n">
-        <v>24014261</v>
+        <v>47583835</v>
       </c>
       <c r="H2" t="n">
-        <v>-0.5904253726566893</v>
+        <v>-0.5805695988984494</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>IOC</t>
+          <t>ETERNAL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>SBILIFE</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>377.45</v>
+        <v>2033.9</v>
       </c>
       <c r="C3" t="n">
-        <v>378.4</v>
+        <v>2050.3</v>
       </c>
       <c r="D3" t="n">
-        <v>372.95</v>
+        <v>2023.8</v>
       </c>
       <c r="E3" t="n">
-        <v>374.3</v>
+        <v>2042</v>
       </c>
       <c r="F3" t="n">
-        <v>2696607</v>
+        <v>580680</v>
       </c>
       <c r="G3" t="n">
-        <v>6352805</v>
+        <v>1240712</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.5755249846327725</v>
+        <v>-0.5319784123954633</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>BPCL</t>
+          <t>SBILIFE</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ASTRAL</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1589</v>
+        <v>1404</v>
       </c>
       <c r="C4" t="n">
-        <v>1604.6</v>
+        <v>1414</v>
       </c>
       <c r="D4" t="n">
-        <v>1559.5</v>
+        <v>1400.5</v>
       </c>
       <c r="E4" t="n">
-        <v>1601</v>
+        <v>1413</v>
       </c>
       <c r="F4" t="n">
-        <v>585825</v>
+        <v>5000042</v>
       </c>
       <c r="G4" t="n">
-        <v>1241019</v>
+        <v>12228083</v>
       </c>
       <c r="H4" t="n">
-        <v>-0.527948403690838</v>
+        <v>-0.5911017287010564</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>ASTRAL</t>
+          <t>ICICIBANK</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>452.35</v>
+        <v>12897</v>
       </c>
       <c r="C5" t="n">
-        <v>455.25</v>
+        <v>12997</v>
       </c>
       <c r="D5" t="n">
-        <v>448.75</v>
+        <v>12861</v>
       </c>
       <c r="E5" t="n">
-        <v>451</v>
+        <v>12949</v>
       </c>
       <c r="F5" t="n">
-        <v>1912866</v>
+        <v>81768</v>
       </c>
       <c r="G5" t="n">
-        <v>3949831</v>
+        <v>178236</v>
       </c>
       <c r="H5" t="n">
-        <v>-0.515709406301181</v>
+        <v>-0.5412374604457012</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>HINDPETRO</t>
+          <t>ULTRACEMCO</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SRF</t>
+          <t>DLF</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2815</v>
+        <v>625.35</v>
       </c>
       <c r="C6" t="n">
-        <v>2841</v>
+        <v>645.3</v>
       </c>
       <c r="D6" t="n">
-        <v>2765.6</v>
+        <v>622</v>
       </c>
       <c r="E6" t="n">
-        <v>2833</v>
+        <v>643.5</v>
       </c>
       <c r="F6" t="n">
-        <v>196550</v>
+        <v>2231253</v>
       </c>
       <c r="G6" t="n">
-        <v>395601</v>
+        <v>4838136</v>
       </c>
       <c r="H6" t="n">
-        <v>-0.5031610132431414</v>
+        <v>-0.5388197024639241</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>SRF</t>
+          <t>DLF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>HAVELLS</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>928.15</v>
+        <v>1404</v>
       </c>
       <c r="C7" t="n">
-        <v>930.9</v>
+        <v>1428.5</v>
       </c>
       <c r="D7" t="n">
-        <v>914.3</v>
+        <v>1396.2</v>
       </c>
       <c r="E7" t="n">
-        <v>919</v>
+        <v>1417.3</v>
       </c>
       <c r="F7" t="n">
-        <v>1221319</v>
+        <v>369629</v>
       </c>
       <c r="G7" t="n">
-        <v>2457834</v>
+        <v>774193</v>
       </c>
       <c r="H7" t="n">
-        <v>-0.5030913397731499</v>
+        <v>-0.5225622034815608</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>FORTIS</t>
+          <t>HAVELLS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SUPREMEIND</t>
+          <t>VEDL</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3827.9</v>
+        <v>669</v>
       </c>
       <c r="C8" t="n">
-        <v>3831.7</v>
+        <v>681.45</v>
       </c>
       <c r="D8" t="n">
-        <v>3745.3</v>
+        <v>665.25</v>
       </c>
       <c r="E8" t="n">
-        <v>3760</v>
+        <v>679.8</v>
       </c>
       <c r="F8" t="n">
-        <v>82044</v>
+        <v>6387272</v>
       </c>
       <c r="G8" t="n">
-        <v>193500</v>
+        <v>15868021</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.576</v>
+        <v>-0.5974751987031023</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>SUPREMEIND</t>
+          <t>VEDL</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>25940</v>
+      </c>
+      <c r="C9" t="n">
+        <v>26375</v>
+      </c>
+      <c r="D9" t="n">
+        <v>25915</v>
+      </c>
+      <c r="E9" t="n">
+        <v>26250</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11713</v>
+      </c>
+      <c r="G9" t="n">
+        <v>27809</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-0.5788054227048797</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>SHREECEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1470</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1494</v>
+      </c>
+      <c r="D10" t="n">
+        <v>1465.2</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1484.8</v>
+      </c>
+      <c r="F10" t="n">
+        <v>217908</v>
+      </c>
+      <c r="G10" t="n">
+        <v>474002</v>
+      </c>
+      <c r="H10" t="n">
+        <v>-0.5402804207577183</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>PIDILITIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>585.95</v>
+      </c>
+      <c r="C11" t="n">
+        <v>596.3</v>
+      </c>
+      <c r="D11" t="n">
+        <v>582.6</v>
+      </c>
+      <c r="E11" t="n">
+        <v>594.5</v>
+      </c>
+      <c r="F11" t="n">
+        <v>4181298</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9424678</v>
+      </c>
+      <c r="H11" t="n">
+        <v>-0.5563457977025846</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>HINDZINC</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>NYKAA</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>270.95</v>
+      </c>
+      <c r="C12" t="n">
+        <v>277.39</v>
+      </c>
+      <c r="D12" t="n">
+        <v>269.24</v>
+      </c>
+      <c r="E12" t="n">
+        <v>275.06</v>
+      </c>
+      <c r="F12" t="n">
+        <v>3543432</v>
+      </c>
+      <c r="G12" t="n">
+        <v>8182107</v>
+      </c>
+      <c r="H12" t="n">
+        <v>-0.5669291540675281</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>NYKAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>MFSL</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>1815.9</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1857.4</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1815.9</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1846.1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>693364</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1588459</v>
+      </c>
+      <c r="H13" t="n">
+        <v>-0.5634989634608133</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>MFSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>79.31999999999999</v>
+      </c>
+      <c r="C14" t="n">
+        <v>80.64</v>
+      </c>
+      <c r="D14" t="n">
+        <v>78.45</v>
+      </c>
+      <c r="E14" t="n">
+        <v>80.27</v>
+      </c>
+      <c r="F14" t="n">
+        <v>15298184</v>
+      </c>
+      <c r="G14" t="n">
+        <v>31361483</v>
+      </c>
+      <c r="H14" t="n">
+        <v>-0.5121983230193546</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>NMDC</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>PETRONET</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>288.3</v>
+      </c>
+      <c r="C15" t="n">
+        <v>295.25</v>
+      </c>
+      <c r="D15" t="n">
+        <v>287.35</v>
+      </c>
+      <c r="E15" t="n">
+        <v>293</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1110180</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2767142</v>
+      </c>
+      <c r="H15" t="n">
+        <v>-0.5987990497054362</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>PETRONET</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>OBEROIRLTY</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>1544.8</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1568.4</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1536.9</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1560.6</v>
+      </c>
+      <c r="F16" t="n">
+        <v>217779</v>
+      </c>
+      <c r="G16" t="n">
+        <v>494872</v>
+      </c>
+      <c r="H16" t="n">
+        <v>-0.5599286280088589</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>OBEROIRLTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>HUDCO</t>
         </is>
       </c>
-      <c r="B9" t="n">
-        <v>201.5</v>
-      </c>
-      <c r="C9" t="n">
-        <v>201.5</v>
-      </c>
-      <c r="D9" t="n">
-        <v>193.78</v>
-      </c>
-      <c r="E9" t="n">
-        <v>195.4</v>
-      </c>
-      <c r="F9" t="n">
+      <c r="B17" t="n">
+        <v>195</v>
+      </c>
+      <c r="C17" t="n">
+        <v>197.34</v>
+      </c>
+      <c r="D17" t="n">
+        <v>193.05</v>
+      </c>
+      <c r="E17" t="n">
+        <v>196.86</v>
+      </c>
+      <c r="F17" t="n">
+        <v>4351756</v>
+      </c>
+      <c r="G17" t="n">
         <v>10052817</v>
       </c>
-      <c r="G9" t="n">
-        <v>22244997</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-0.5480863854465793</v>
-      </c>
-      <c r="I9" t="inlineStr">
+      <c r="H17" t="n">
+        <v>-0.5671107909355159</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>HUDCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ASHOKLEY</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>204.95</v>
+      </c>
+      <c r="C18" t="n">
+        <v>206.89</v>
+      </c>
+      <c r="D18" t="n">
+        <v>203</v>
+      </c>
+      <c r="E18" t="n">
+        <v>205.5</v>
+      </c>
+      <c r="F18" t="n">
+        <v>11066053</v>
+      </c>
+      <c r="G18" t="n">
+        <v>26832686</v>
+      </c>
+      <c r="H18" t="n">
+        <v>-0.5875905602592301</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>ASHOKLEY</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>HINDPETRO</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>448</v>
+      </c>
+      <c r="C19" t="n">
+        <v>452.6</v>
+      </c>
+      <c r="D19" t="n">
+        <v>445</v>
+      </c>
+      <c r="E19" t="n">
+        <v>451.9</v>
+      </c>
+      <c r="F19" t="n">
+        <v>879388</v>
+      </c>
+      <c r="G19" t="n">
+        <v>1912866</v>
+      </c>
+      <c r="H19" t="n">
+        <v>-0.5402772593584705</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>HINDPETRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>COLPAL</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>2120.6</v>
+      </c>
+      <c r="C20" t="n">
+        <v>2128.3</v>
+      </c>
+      <c r="D20" t="n">
+        <v>2100.7</v>
+      </c>
+      <c r="E20" t="n">
+        <v>2117</v>
+      </c>
+      <c r="F20" t="n">
+        <v>154505</v>
+      </c>
+      <c r="G20" t="n">
+        <v>374088</v>
+      </c>
+      <c r="H20" t="n">
+        <v>-0.5869822073950515</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>COLPAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>TATAELXSI</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>4824</v>
+      </c>
+      <c r="C21" t="n">
+        <v>4845</v>
+      </c>
+      <c r="D21" t="n">
+        <v>4750</v>
+      </c>
+      <c r="E21" t="n">
+        <v>4811</v>
+      </c>
+      <c r="F21" t="n">
+        <v>215518</v>
+      </c>
+      <c r="G21" t="n">
+        <v>441804</v>
+      </c>
+      <c r="H21" t="n">
+        <v>-0.5121863993988285</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>TATAELXSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>SAIL</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>158</v>
+      </c>
+      <c r="C22" t="n">
+        <v>160.14</v>
+      </c>
+      <c r="D22" t="n">
+        <v>157.25</v>
+      </c>
+      <c r="E22" t="n">
+        <v>158.8</v>
+      </c>
+      <c r="F22" t="n">
+        <v>8429730</v>
+      </c>
+      <c r="G22" t="n">
+        <v>19899685</v>
+      </c>
+      <c r="H22" t="n">
+        <v>-0.5763887719830741</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>SAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TIINDIA</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>2490</v>
+      </c>
+      <c r="C23" t="n">
+        <v>2524</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2479</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2491</v>
+      </c>
+      <c r="F23" t="n">
+        <v>138570</v>
+      </c>
+      <c r="G23" t="n">
+        <v>315365</v>
+      </c>
+      <c r="H23" t="n">
+        <v>-0.5606043790528435</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>TIINDIA</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PAYTM</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>1120.5</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1126.9</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1101.8</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1122</v>
+      </c>
+      <c r="F24" t="n">
+        <v>2605903</v>
+      </c>
+      <c r="G24" t="n">
+        <v>6319748</v>
+      </c>
+      <c r="H24" t="n">
+        <v>-0.5876571344300437</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>PAYTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ICICIPRULI</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>643</v>
+      </c>
+      <c r="C25" t="n">
+        <v>643.75</v>
+      </c>
+      <c r="D25" t="n">
+        <v>633.7</v>
+      </c>
+      <c r="E25" t="n">
+        <v>639.75</v>
+      </c>
+      <c r="F25" t="n">
+        <v>295460</v>
+      </c>
+      <c r="G25" t="n">
+        <v>711887</v>
+      </c>
+      <c r="H25" t="n">
+        <v>-0.5849622201276327</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>ICICIPRULI</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PIIND</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>3089.7</v>
+      </c>
+      <c r="C26" t="n">
+        <v>3167.4</v>
+      </c>
+      <c r="D26" t="n">
+        <v>3021.7</v>
+      </c>
+      <c r="E26" t="n">
+        <v>3050</v>
+      </c>
+      <c r="F26" t="n">
+        <v>600277</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1327261</v>
+      </c>
+      <c r="H26" t="n">
+        <v>-0.5477325107872528</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>PIIND</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>PNBHOUSING</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>832</v>
+      </c>
+      <c r="C27" t="n">
+        <v>853.8</v>
+      </c>
+      <c r="D27" t="n">
+        <v>830.15</v>
+      </c>
+      <c r="E27" t="n">
+        <v>845</v>
+      </c>
+      <c r="F27" t="n">
+        <v>503367</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1057628</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.5240604446932192</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>PNBHOUSING</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>AMBER</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>7760</v>
+      </c>
+      <c r="C28" t="n">
+        <v>7812.5</v>
+      </c>
+      <c r="D28" t="n">
+        <v>7687.5</v>
+      </c>
+      <c r="E28" t="n">
+        <v>7757</v>
+      </c>
+      <c r="F28" t="n">
+        <v>163902</v>
+      </c>
+      <c r="G28" t="n">
+        <v>351861</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.5341853743381619</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>AMBER</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RBLBANK</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>312.35</v>
+      </c>
+      <c r="C29" t="n">
+        <v>315.3</v>
+      </c>
+      <c r="D29" t="n">
+        <v>310.25</v>
+      </c>
+      <c r="E29" t="n">
+        <v>313.6</v>
+      </c>
+      <c r="F29" t="n">
+        <v>1778001</v>
+      </c>
+      <c r="G29" t="n">
+        <v>3835217</v>
+      </c>
+      <c r="H29" t="n">
+        <v>-0.536401460464949</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>RBLBANK</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>IIFL</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>505.1</v>
+      </c>
+      <c r="C30" t="n">
+        <v>512.95</v>
+      </c>
+      <c r="D30" t="n">
+        <v>496.15</v>
+      </c>
+      <c r="E30" t="n">
+        <v>507.55</v>
+      </c>
+      <c r="F30" t="n">
+        <v>965895</v>
+      </c>
+      <c r="G30" t="n">
+        <v>2280434</v>
+      </c>
+      <c r="H30" t="n">
+        <v>-0.5764424666532774</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>IIFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>CYIENT</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C31" t="n">
+        <v>1002.1</v>
+      </c>
+      <c r="D31" t="n">
+        <v>985</v>
+      </c>
+      <c r="E31" t="n">
+        <v>992</v>
+      </c>
+      <c r="F31" t="n">
+        <v>167975</v>
+      </c>
+      <c r="G31" t="n">
+        <v>370990</v>
+      </c>
+      <c r="H31" t="n">
+        <v>-0.5472249925874013</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>CYIENT</t>
         </is>
       </c>
     </row>
@@ -751,7 +1477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -804,528 +1530,297 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>265</v>
+        <v>1128.5</v>
       </c>
       <c r="C2" t="n">
-        <v>267.25</v>
+        <v>1141.8</v>
       </c>
       <c r="D2" t="n">
-        <v>262.85</v>
+        <v>1117.1</v>
       </c>
       <c r="E2" t="n">
-        <v>263.85</v>
+        <v>1138.8</v>
       </c>
       <c r="F2" t="n">
-        <v>12222314</v>
+        <v>780629</v>
       </c>
       <c r="G2" t="n">
-        <v>8681589</v>
+        <v>525887</v>
       </c>
       <c r="H2" t="n">
-        <v>0.4078429651530383</v>
+        <v>0.4844044443007718</v>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>JIOFIN</t>
+          <t>TATACONSUM</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ADANIGREEN</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>913</v>
+        <v>949.5</v>
       </c>
       <c r="C3" t="n">
-        <v>928.2</v>
+        <v>999</v>
       </c>
       <c r="D3" t="n">
-        <v>901</v>
+        <v>936.45</v>
       </c>
       <c r="E3" t="n">
-        <v>903.9</v>
+        <v>991.8</v>
       </c>
       <c r="F3" t="n">
-        <v>50188359</v>
+        <v>4171950</v>
       </c>
       <c r="G3" t="n">
-        <v>33872203</v>
+        <v>2943844</v>
       </c>
       <c r="H3" t="n">
-        <v>0.4816975146257833</v>
+        <v>0.4171776765344903</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>HDFCBANK</t>
+          <t>ADANIGREEN</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>348.1</v>
+        <v>5980</v>
       </c>
       <c r="C4" t="n">
-        <v>348.5</v>
+        <v>6134</v>
       </c>
       <c r="D4" t="n">
-        <v>339.8</v>
+        <v>5964.5</v>
       </c>
       <c r="E4" t="n">
-        <v>346</v>
+        <v>6100</v>
       </c>
       <c r="F4" t="n">
-        <v>8552636</v>
+        <v>255274</v>
       </c>
       <c r="G4" t="n">
-        <v>5630751</v>
+        <v>159821</v>
       </c>
       <c r="H4" t="n">
-        <v>0.5189156828280987</v>
+        <v>0.5972494227917483</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>RECLTD</t>
+          <t>BRITANNIA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>LTF</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>479</v>
+        <v>284</v>
       </c>
       <c r="C5" t="n">
-        <v>479</v>
+        <v>295.45</v>
       </c>
       <c r="D5" t="n">
-        <v>468.85</v>
+        <v>281.2</v>
       </c>
       <c r="E5" t="n">
-        <v>471.4</v>
+        <v>295.1</v>
       </c>
       <c r="F5" t="n">
-        <v>1171877</v>
+        <v>6790971</v>
       </c>
       <c r="G5" t="n">
-        <v>831728</v>
+        <v>4322331</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4089666333224323</v>
+        <v>0.5711362688327202</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>JSWENERGY</t>
+          <t>LTF</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>INDIANB</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>36415</v>
+        <v>869</v>
       </c>
       <c r="C6" t="n">
-        <v>36420</v>
+        <v>892.4</v>
       </c>
       <c r="D6" t="n">
-        <v>35600</v>
+        <v>863.1</v>
       </c>
       <c r="E6" t="n">
-        <v>35700</v>
+        <v>890</v>
       </c>
       <c r="F6" t="n">
-        <v>13848</v>
+        <v>1290153</v>
       </c>
       <c r="G6" t="n">
-        <v>9373</v>
+        <v>877486</v>
       </c>
       <c r="H6" t="n">
-        <v>0.4774351861730503</v>
+        <v>0.4702832865709539</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>BOSCHLTD</t>
+          <t>INDIANB</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>IRB</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>13250</v>
+        <v>44</v>
       </c>
       <c r="C7" t="n">
-        <v>13300</v>
+        <v>44</v>
       </c>
       <c r="D7" t="n">
-        <v>12935</v>
+        <v>41.88</v>
       </c>
       <c r="E7" t="n">
-        <v>12965</v>
+        <v>42.21</v>
       </c>
       <c r="F7" t="n">
-        <v>90669</v>
+        <v>11141730</v>
       </c>
       <c r="G7" t="n">
-        <v>60892</v>
+        <v>7597646</v>
       </c>
       <c r="H7" t="n">
-        <v>0.4890133350850687</v>
+        <v>0.466471325460544</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>SOLARINDS</t>
+          <t>IRB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>MCX</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>641.6</v>
+        <v>2240</v>
       </c>
       <c r="C8" t="n">
-        <v>641.6</v>
+        <v>2358.2</v>
       </c>
       <c r="D8" t="n">
-        <v>623.55</v>
+        <v>2168</v>
       </c>
       <c r="E8" t="n">
-        <v>626.95</v>
+        <v>2350</v>
       </c>
       <c r="F8" t="n">
-        <v>4838136</v>
+        <v>5065061</v>
       </c>
       <c r="G8" t="n">
-        <v>3109096</v>
+        <v>3459271</v>
       </c>
       <c r="H8" t="n">
-        <v>0.5561230659973189</v>
+        <v>0.4641989598386481</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>DLF</t>
+          <t>MCX</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>GRANULES</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1149.1</v>
+        <v>560.6</v>
       </c>
       <c r="C9" t="n">
-        <v>1157.4</v>
+        <v>567.3</v>
       </c>
       <c r="D9" t="n">
-        <v>1126.8</v>
+        <v>556</v>
       </c>
       <c r="E9" t="n">
-        <v>1157</v>
+        <v>564</v>
       </c>
       <c r="F9" t="n">
-        <v>1682470</v>
+        <v>522642</v>
       </c>
       <c r="G9" t="n">
-        <v>1090045</v>
+        <v>366379</v>
       </c>
       <c r="H9" t="n">
-        <v>0.5434867367860959</v>
+        <v>0.4265064318642717</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AUROPHARMA</t>
+          <t>GRANULES</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
+          <t>MANAPPURAM</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>4425</v>
+        <v>303.25</v>
       </c>
       <c r="C10" t="n">
-        <v>4491.9</v>
+        <v>306</v>
       </c>
       <c r="D10" t="n">
-        <v>4395.2</v>
+        <v>295.35</v>
       </c>
       <c r="E10" t="n">
-        <v>4412</v>
+        <v>302.8</v>
       </c>
       <c r="F10" t="n">
-        <v>512643</v>
+        <v>7805766</v>
       </c>
       <c r="G10" t="n">
-        <v>360796</v>
+        <v>4916102</v>
       </c>
       <c r="H10" t="n">
-        <v>0.4208666393197264</v>
+        <v>0.5877957780371522</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>CUMMINSIND</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>MPHASIS</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>2387.6</v>
-      </c>
-      <c r="C11" t="n">
-        <v>2501.2</v>
-      </c>
-      <c r="D11" t="n">
-        <v>2355.2</v>
-      </c>
-      <c r="E11" t="n">
-        <v>2452.5</v>
-      </c>
-      <c r="F11" t="n">
-        <v>1725163</v>
-      </c>
-      <c r="G11" t="n">
-        <v>1136104</v>
-      </c>
-      <c r="H11" t="n">
-        <v>0.5184903846830924</v>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>MPHASIS</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>LUPIN</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>2210</v>
-      </c>
-      <c r="C12" t="n">
-        <v>2219.2</v>
-      </c>
-      <c r="D12" t="n">
-        <v>2160</v>
-      </c>
-      <c r="E12" t="n">
-        <v>2194</v>
-      </c>
-      <c r="F12" t="n">
-        <v>1126141</v>
-      </c>
-      <c r="G12" t="n">
-        <v>804229</v>
-      </c>
-      <c r="H12" t="n">
-        <v>0.4002740512963348</v>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>LUPIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>DIXON</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>11500</v>
-      </c>
-      <c r="C13" t="n">
-        <v>11548</v>
-      </c>
-      <c r="D13" t="n">
-        <v>11250</v>
-      </c>
-      <c r="E13" t="n">
-        <v>11398</v>
-      </c>
-      <c r="F13" t="n">
-        <v>446533</v>
-      </c>
-      <c r="G13" t="n">
-        <v>288312</v>
-      </c>
-      <c r="H13" t="n">
-        <v>0.5487839562695969</v>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>DIXON</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>BANKINDIA</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>164.1</v>
-      </c>
-      <c r="C14" t="n">
-        <v>164.45</v>
-      </c>
-      <c r="D14" t="n">
-        <v>161.26</v>
-      </c>
-      <c r="E14" t="n">
-        <v>161.69</v>
-      </c>
-      <c r="F14" t="n">
-        <v>8120034</v>
-      </c>
-      <c r="G14" t="n">
-        <v>5243794</v>
-      </c>
-      <c r="H14" t="n">
-        <v>0.5485036216144265</v>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>BANKINDIA</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>BSE</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>3100</v>
-      </c>
-      <c r="C15" t="n">
-        <v>3127</v>
-      </c>
-      <c r="D15" t="n">
-        <v>3017.9</v>
-      </c>
-      <c r="E15" t="n">
-        <v>3023.9</v>
-      </c>
-      <c r="F15" t="n">
-        <v>3885000</v>
-      </c>
-      <c r="G15" t="n">
-        <v>2525871</v>
-      </c>
-      <c r="H15" t="n">
-        <v>0.5380832987907933</v>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>BSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CROMPTON</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>264</v>
-      </c>
-      <c r="C16" t="n">
-        <v>269.85</v>
-      </c>
-      <c r="D16" t="n">
-        <v>255.9</v>
-      </c>
-      <c r="E16" t="n">
-        <v>266.8</v>
-      </c>
-      <c r="F16" t="n">
-        <v>4504154</v>
-      </c>
-      <c r="G16" t="n">
-        <v>3035533</v>
-      </c>
-      <c r="H16" t="n">
-        <v>0.4838099272845988</v>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>CROMPTON</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>CDSL</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>1350</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1359</v>
-      </c>
-      <c r="D17" t="n">
-        <v>1321.1</v>
-      </c>
-      <c r="E17" t="n">
-        <v>1335.6</v>
-      </c>
-      <c r="F17" t="n">
-        <v>1663043</v>
-      </c>
-      <c r="G17" t="n">
-        <v>1133736</v>
-      </c>
-      <c r="H17" t="n">
-        <v>0.4668697121728515</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>CDSL</t>
+          <t>MANAPPURAM</t>
         </is>
       </c>
     </row>

</xml_diff>